<commit_message>
prepare for a big revision
</commit_message>
<xml_diff>
--- a/计分.xlsx
+++ b/计分.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\life\board_game\project_six_dynasty\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B771923D-0E4A-42A4-AAD3-30B736AA9A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906F756D-4909-4430-AFFC-AC91559021BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8AF991C0-2FFC-4B9D-8DFA-610AA56EBD09}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>计分</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -146,6 +146,22 @@
   </si>
   <si>
     <t>紫色/王导</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v0.2_0521</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>蓝色/桓温</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>绿色/chijian</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>紫色/祖逖</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -530,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42E67ED8-6937-492E-8350-3FCD992CF871}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
@@ -837,16 +853,12 @@
       <c r="M11">
         <v>4</v>
       </c>
-      <c r="N11">
-        <f>CEILING(L$10/10,1)*M11</f>
-        <v>32</v>
-      </c>
       <c r="O11">
         <v>16</v>
       </c>
       <c r="P11">
         <f t="shared" si="2"/>
-        <v>127</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -927,6 +939,164 @@
       <c r="P13">
         <f t="shared" si="2"/>
         <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>12</v>
+      </c>
+      <c r="H16">
+        <v>5</v>
+      </c>
+      <c r="I16">
+        <v>6</v>
+      </c>
+      <c r="K16">
+        <v>110</v>
+      </c>
+      <c r="P16">
+        <f t="shared" ref="P16:P20" si="4">SUM(B16:O16)</f>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="H17">
+        <v>12</v>
+      </c>
+      <c r="I17">
+        <v>14</v>
+      </c>
+      <c r="K17">
+        <v>72</v>
+      </c>
+      <c r="L17">
+        <f>SUM(H17:K17)</f>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18">
+        <v>8</v>
+      </c>
+      <c r="I18">
+        <v>16</v>
+      </c>
+      <c r="J18">
+        <v>19</v>
+      </c>
+      <c r="K18">
+        <v>70</v>
+      </c>
+      <c r="M18">
+        <v>4</v>
+      </c>
+      <c r="N18">
+        <f>CEILING(L$17/10,1)*M11</f>
+        <v>40</v>
+      </c>
+      <c r="O18">
+        <v>30</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="4"/>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>12</v>
+      </c>
+      <c r="H19">
+        <v>5</v>
+      </c>
+      <c r="I19">
+        <v>10</v>
+      </c>
+      <c r="J19">
+        <v>19</v>
+      </c>
+      <c r="K19">
+        <v>59</v>
+      </c>
+      <c r="M19">
+        <v>4</v>
+      </c>
+      <c r="N19">
+        <f>CEILING(L$17/10,1)*M12</f>
+        <v>40</v>
+      </c>
+      <c r="O19">
+        <v>14</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="4"/>
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>18</v>
+      </c>
+      <c r="G20">
+        <v>9</v>
+      </c>
+      <c r="H20">
+        <v>7</v>
+      </c>
+      <c r="I20">
+        <v>10</v>
+      </c>
+      <c r="J20">
+        <v>20</v>
+      </c>
+      <c r="K20">
+        <v>55</v>
+      </c>
+      <c r="M20">
+        <v>4</v>
+      </c>
+      <c r="N20">
+        <f>CEILING(L$17/10,1)*M13</f>
+        <v>40</v>
+      </c>
+      <c r="O20">
+        <v>18</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="4"/>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>